<commit_message>
chore(bkm): verimlilik Excel tek dosyada toplandı (v2/v3 kopyaları kaldırıldı)
Dosya kilitli olduğu için v2/v3 adlarıyla üretilmişti; kullanıcı kapattı → içerik
kanonik verimlilik-2026.xlsx'e yazıldı (8 sayfa, Sunum ilk sayfa). Kopyalar silindi:
aynı raporun üç adı karışıklık üretiyor, script her çalıştırmada kanonik adı üretir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/briefings/sezon-kadro-20260902/verimlilik-2026.xlsx
+++ b/briefings/sezon-kadro-20260902/verimlilik-2026.xlsx
@@ -7,11 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ozet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magaza" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yillar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oca-Agu" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yontem" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sunum" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magaza" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kadro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bolum" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yillar" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oca-Agu" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yontem" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +23,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="+0.0%;-0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="+0;-0;0"/>
+  <numFmts count="9">
+    <numFmt numFmtId="164" formatCode="+#,##0;-#,##0;0"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="168" formatCode="+0;-0;0"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="+0 kişi;-0 kişi"/>
+    <numFmt numFmtId="171" formatCode="+0,0%"/>
+    <numFmt numFmtId="172" formatCode="0,0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,7 +53,6 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -58,12 +65,41 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F5B57"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F7A4D"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00444444"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F5B57"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +109,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E30622"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F5B57"/>
       </patternFill>
     </fill>
     <fill>
@@ -112,43 +153,79 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -795,10 +872,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A2:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Sezon 2026 — kadro mu büyüdü, iş mi büyüdü?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Beş mağaza kadrosu · üç POS mağazası iş hacmi · 2025 ile aynı takvim dönemi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Kadro farkı sezon başlamadan ÖNCE oluştu.</t>
+        </is>
+      </c>
+      <c r="C5" s="5">
+        <f>'Ozet'!D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>30 Haziran'da kadrolu personel 139'dan 153'e çıkmıştı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Sezon boyunca kadro büyümedi, KÜÇÜLDÜ.</t>
+        </is>
+      </c>
+      <c r="C7" s="5">
+        <f>'Ozet'!C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>1 Temmuz – 31 Ağustos: kadrolu 153 → 149. Geçen yıl da aynı yönde (−4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Sezonluk personel geçen yıldan AZ.</t>
+        </is>
+      </c>
+      <c r="C9" s="5">
+        <f>'Ozet'!D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>31 Ağustos'ta çalışan sezonluk: 65 → 62 kişi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Aynı dönemde elleçlenen ürün adedi %35 arttı.</t>
+        </is>
+      </c>
+      <c r="C11" s="7">
+        <f>'Ozet'!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>574.718 → 775.192 adet. Adet enflasyondan etkilenmez — fiilen kasadan geçen, rafa dizilen mal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Ciro %71 arttı.</t>
+        </is>
+      </c>
+      <c r="C13" s="7">
+        <f>'Ozet'!E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>71,8 milyon → 122,6 milyon ₺ (KDV dahil, iadeler düşülmüş).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>KİŞİ BAŞINA düşen iş de arttı.</t>
+        </is>
+      </c>
+      <c r="C15" s="7">
+        <f>'Ozet'!E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Kişi başı ürün 4.019 → 4.845 adet; günlük 71,8 → 86,5 adet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>İş hacmi, kadronun yaklaşık 3 KATI hızla büyüdü.</t>
+        </is>
+      </c>
+      <c r="C17" s="8">
+        <f>'Ozet'!B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Ürün adedi +%34,9 · kadro +%11,9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Artış yönetimde değil, RAFIN ÖNÜNDE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Yönetim +0 · Mal Kabul +0 · İdari İşler +0. Artış: Yardımcı Kitap +6 · Kırtasiye +3 · Kasa +2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Büyüme kurumsaldan gelmedi, mağazadan geldi.</t>
+        </is>
+      </c>
+      <c r="C21" s="7">
+        <f>'Oca-Agu'!G4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Sınav Okulları Ocak–Ağustos cirosu −%22,4 küçüldü; mağaza tarafı +%54,9 büyüdü.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="9" t="n"/>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>TEK CÜMLE: Kadro farkı 1 Temmuz'dan önce kurulmuştu; sezon içinde kadro küçülürken iş hacmi %35 büyüdü, kişi başına düşen iş %21 arttı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Rakamların kaynağı ve kontrolü: Ozet · Magaza · Kadro · Bolum · Yillar · Oca-Agu · Yontem sayfaları. Kadro = Zirve İK (İK'nın kendi karşılaştırma raporuyla birebir), iş hacmi = DerinSIS mağaza satışı (Sınav hariç).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -806,337 +1134,511 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ayni kadro, daha cok is — uc POS magazasi (okul-hizali pencere, 56 gun)</t>
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Ayni kadro, daha cok is — kapsamlar AYRI etiketli, altta kopru kontrolu</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Olcu</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Fark</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Degisim</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Kadro — 31.08 (kisi)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>143</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="D4" s="4">
-        <f>C4-B4</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>IF(B4=0,"",C4/B4-1)</f>
-        <v/>
-      </c>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>KAPSAM A — UC POS MAGAZASI (FSM · Ozluce · Ist. Yolu) · is hacmi YALNIZ burada olculebilir</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Urun adedi (elleclenen)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Kadrolu — 31.08</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>96</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>111</v>
+      </c>
+      <c r="D5" s="18">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="19">
+        <f>IF(B5=0,"",C5/B5-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Sezonluk — 31.08</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>47</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="D6" s="18">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="19">
+        <f>IF(B6=0,"",C6/B6-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20">
+        <f> TOPLAM KADRO — 31.08 (kisi)</f>
+        <v/>
+      </c>
+      <c r="B7" s="21">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="21">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="22">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="23">
+        <f>C7/B7-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urun adedi (elleclenen) — 56 gun</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
         <v>574717.7</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C8" s="17" t="n">
         <v>775191.55</v>
       </c>
-      <c r="D5" s="4">
-        <f>C5-B5</f>
-        <v/>
-      </c>
-      <c r="E5" s="5">
-        <f>IF(B5=0,"",C5/B5-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Ciro — KDV haric (TL)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>66929723.56999837</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>114687785.5800005</v>
-      </c>
-      <c r="D6" s="4">
-        <f>C6-B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>IF(B6=0,"",C6/B6-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Ciro — KDV dahil (TL)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>71837429.11999327</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>122601380.8499953</v>
-      </c>
-      <c r="D7" s="4">
-        <f>C7-B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>IF(B7=0,"",C7/B7-1)</f>
+      <c r="D8" s="18">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>IF(B8=0,"",C8/B8-1)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>KISI BASI — asil olcu</t>
-        </is>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ciro — KDV haric (TL)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>66929723.56999852</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>114687785.58</v>
+      </c>
+      <c r="D9" s="18">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>IF(B9=0,"",C9/B9-1)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Urun adedi / kisi</t>
-        </is>
-      </c>
-      <c r="B10" s="7">
-        <f>B5/B4</f>
-        <v/>
-      </c>
-      <c r="C10" s="7">
-        <f>C5/C4</f>
-        <v/>
-      </c>
-      <c r="D10" s="7">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ciro — KDV dahil (TL)</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>71837429.11999343</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>122601380.8499947</v>
+      </c>
+      <c r="D10" s="18">
         <f>C10-B10</f>
         <v/>
       </c>
-      <c r="E10" s="8">
-        <f>C10/B10-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Urun adedi / kisi / gun</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>B5/B4/56</f>
-        <v/>
-      </c>
-      <c r="C11" s="9">
-        <f>C5/C4/56</f>
-        <v/>
-      </c>
-      <c r="D11" s="9">
-        <f>C11-B11</f>
-        <v/>
-      </c>
-      <c r="E11" s="8">
-        <f>C11/B11-1</f>
+      <c r="E10" s="19">
+        <f>IF(B10=0,"",C10/B10-1)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Ciro (KDV haric) / kisi (TL)</t>
-        </is>
-      </c>
-      <c r="B12" s="7">
-        <f>B6/B4</f>
-        <v/>
-      </c>
-      <c r="C12" s="7">
-        <f>C6/C4</f>
-        <v/>
-      </c>
-      <c r="D12" s="7">
-        <f>C12-B12</f>
-        <v/>
-      </c>
-      <c r="E12" s="8">
-        <f>C12/B12-1</f>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>KISI BASI — asil olcu · kapsam A toplam kadrosuna bolunur (satir 7)</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urun adedi / kisi</t>
+        </is>
+      </c>
+      <c r="B13" s="24">
+        <f>B8/B7</f>
+        <v/>
+      </c>
+      <c r="C13" s="24">
+        <f>C8/C7</f>
+        <v/>
+      </c>
+      <c r="D13" s="24">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="25">
+        <f>C13/B13-1</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Is buyumesi kadro buyumesinin kac kati</t>
-        </is>
-      </c>
-      <c r="B14" s="11">
-        <f>E5/E4</f>
-        <v/>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>urun adedi / kadro</t>
-        </is>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urun adedi / kisi / gun</t>
+        </is>
+      </c>
+      <c r="B14" s="26">
+        <f>B8/B7/56</f>
+        <v/>
+      </c>
+      <c r="C14" s="26">
+        <f>C8/C7/56</f>
+        <v/>
+      </c>
+      <c r="D14" s="26">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="25">
+        <f>C14/B14-1</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ayni oran ciro ile</t>
-        </is>
-      </c>
-      <c r="B15" s="13">
-        <f>E6/E4</f>
-        <v/>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>ciro (KDV haric) / kadro</t>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ciro (KDV haric) / kisi (TL)</t>
+        </is>
+      </c>
+      <c r="B15" s="24">
+        <f>B9/B7</f>
+        <v/>
+      </c>
+      <c r="C15" s="24">
+        <f>C9/C7</f>
+        <v/>
+      </c>
+      <c r="D15" s="24">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="25">
+        <f>C15/B15-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Is buyumesi kadro buyumesinin kac kati (adet ÷ kadro)</t>
+        </is>
+      </c>
+      <c r="B16" s="27">
+        <f>E8/E7</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>adet degisimi ÷ kadro degisimi</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>BES MAGAZA KADRO HAREKETI (POS'ta olmayan Heykel + Sura dahil)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Kadrolu — taban 30.06</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ayni oran ciro ile (ciro ÷ kadro)</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
+        <f>E9/E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>KAPSAM B — BES MAGAZA (+ Heykel, Sura: POS raporlamasinda YOK -&gt; is hacmi olculemez)</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Kadrolu — TABAN 30.06 (sezon oncesi kurulu kadro)</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n">
         <v>139</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C20" s="21" t="n">
         <v>153</v>
       </c>
-      <c r="D18" s="14">
-        <f>C18-B18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Kadrolu — kesim 31.08</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
+      <c r="D20" s="29">
+        <f>C20-B20</f>
+        <v/>
+      </c>
+      <c r="E20" s="19">
+        <f>IF(B20=0,"",C20/B20-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Kadrolu — KESIM 31.08</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="n">
         <v>135</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C21" s="17" t="n">
         <v>149</v>
       </c>
-      <c r="D19" s="14">
-        <f>C19-B19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Sezonluk — kesim 31.08</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
+      <c r="D21" s="18">
+        <f>C21-B21</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>IF(B21=0,"",C21/B21-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Sezon ici kadrolu degisim (kesim - taban)</t>
+        </is>
+      </c>
+      <c r="B22" s="30">
+        <f>B21-B20</f>
+        <v/>
+      </c>
+      <c r="C22" s="30">
+        <f>C21-C20</f>
+        <v/>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>iki yilda da -4: sezon icinde kadro BUYUMEDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Sezonluk — 31.08</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="n">
         <v>65</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C23" s="17" t="n">
         <v>62</v>
       </c>
-      <c r="D20" s="14">
-        <f>C20-B20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Toplam — kesim 31.08</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>211</v>
-      </c>
-      <c r="D21" s="14">
-        <f>C21-B21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Sezon ici kadrolu degisim (taban -&gt; kesim)</t>
-        </is>
-      </c>
-      <c r="B22" s="14">
-        <f>B19-B18</f>
-        <v/>
-      </c>
-      <c r="C22" s="15">
-        <f>C19-C18</f>
-        <v/>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>sezon icinde kadro BUYUMEDI</t>
-        </is>
+      <c r="D23" s="18">
+        <f>C23-B23</f>
+        <v/>
+      </c>
+      <c r="E23" s="19">
+        <f>IF(B23=0,"",C23/B23-1)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Kadro farki 1 Temmuz'dan ONCE olustu: kadrolu taban 30.06'da 139 -&gt; 153. Sezon icinde (1 Tem - 31 Agu) kadro kucumustu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Kisi basi satirlar ve tum yuzdeler Excel FORMULUDUR — ham rakami degistirin, oran kendini gunceller.</t>
+          <t xml:space="preserve">   = Toplam kadro — 31.08</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>211</v>
+      </c>
+      <c r="D24" s="18">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+      <c r="E24" s="19">
+        <f>IF(B24=0,"",C24/B24-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>KOPRU — A ile B nasil bagli (KONTROL satiri 0 olmali)</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Kapsam A toplam kadro (31.08)</t>
+        </is>
+      </c>
+      <c r="B27" s="17">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C27" s="17">
+        <f>C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   + Heykel + Sura (kadrolu + sezonluk)</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="n">
+        <v>57</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="D28" s="18">
+        <f>C28-B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = Kapsam B toplam kadro (hesap)</t>
+        </is>
+      </c>
+      <c r="B29" s="21">
+        <f>B27+B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="21">
+        <f>C27+C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   KONTROL: hesap - B blogundaki toplam (0 OLMALI)</t>
+        </is>
+      </c>
+      <c r="B30" s="31">
+        <f>B29-B24</f>
+        <v/>
+      </c>
+      <c r="C30" s="31">
+        <f>C29-C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>NEDEN IKI KAPSAM: is hacmi (adet/ciro) yalniz POS raporlamasi olan UC magazada olculebilir;</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   kadro hareketi ise bes magazanin tamaminda anlamli. Karismasin diye bloklar ayri + kopru var.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>NEDEN IKI TARIH: 30.06 = sezon baslamadan onceki kurulu kadro (+14 farki BURADA olustu),</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   31.08 = sezon zirvesindeki fiili kadro. Ayni yilin iki farkli gunu; birbirinin yerine gecmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>Kadrolu = Kadro &lt;&gt; 'SEZONLUK' · Sezonluk = Kadro = 'SEZONLUK' · Toplam = ikisinin toplami.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>Tum yuzde / oran / kopru satirlari Excel FORMULU — ham rakami degistir, hepsi kendini gunceller.</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1176,330 +1678,330 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Magaza bazinda kisi basi is — okul-hizali pencere (56 gun, Sinav haric)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Magaza</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Kadro 2025</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Kadro 2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Kadro Δ%</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Urun adedi 2025</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>Urun adedi 2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Adet Δ%</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>Adet/kisi 2025</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>Adet/kisi 2026</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Adet/kisi Δ%</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Adet/kisi/gun 2025</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L3" s="13" t="inlineStr">
         <is>
           <t>Adet/kisi/gun 2026</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M3" s="13" t="inlineStr">
         <is>
           <t>Ciro 2025 (KDV haric)</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" s="13" t="inlineStr">
         <is>
           <t>Ciro 2026 (KDV haric)</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O3" s="13" t="inlineStr">
         <is>
           <t>Ciro Δ%</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="P3" s="13" t="inlineStr">
         <is>
           <t>Ciro/kisi 2025</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="Q3" s="13" t="inlineStr">
         <is>
           <t>Ciro/kisi 2026</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="R3" s="13" t="inlineStr">
         <is>
           <t>Ciro/kisi Δ%</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="S3" s="13" t="inlineStr">
         <is>
           <t>Is / kadro (kac kat)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>İst. Yolu</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="17" t="n">
         <v>61</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="19">
         <f>C4/B4-1</f>
         <v/>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="17" t="n">
         <v>173398</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="17" t="n">
         <v>258168.5</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="19">
         <f>F4/E4-1</f>
         <v/>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="17">
         <f>E4/B4</f>
         <v/>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="17">
         <f>F4/C4</f>
         <v/>
       </c>
-      <c r="J4" s="17">
+      <c r="J4" s="33">
         <f>I4/H4-1</f>
         <v/>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="34">
         <f>E4/B4/56</f>
         <v/>
       </c>
-      <c r="L4" s="18">
+      <c r="L4" s="34">
         <f>F4/C4/56</f>
         <v/>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>20455158.42999977</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>40444611.76999984</v>
-      </c>
-      <c r="O4" s="5">
+      <c r="M4" s="17" t="n">
+        <v>20455158.42999981</v>
+      </c>
+      <c r="N4" s="17" t="n">
+        <v>40444611.76999976</v>
+      </c>
+      <c r="O4" s="19">
         <f>N4/M4-1</f>
         <v/>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="17">
         <f>M4/B4</f>
         <v/>
       </c>
-      <c r="Q4" s="4">
+      <c r="Q4" s="17">
         <f>N4/C4</f>
         <v/>
       </c>
-      <c r="R4" s="17">
+      <c r="R4" s="33">
         <f>Q4/P4-1</f>
         <v/>
       </c>
-      <c r="S4" s="19">
+      <c r="S4" s="35">
         <f>G4/D4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Özlüce</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="17" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="17" t="n">
         <v>54</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="19">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="17" t="n">
         <v>230764.7</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="17" t="n">
         <v>301250.05</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="19">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="17">
         <f>E5/B5</f>
         <v/>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="17">
         <f>F5/C5</f>
         <v/>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="33">
         <f>I5/H5-1</f>
         <v/>
       </c>
-      <c r="K5" s="18">
+      <c r="K5" s="34">
         <f>E5/B5/56</f>
         <v/>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="34">
         <f>F5/C5/56</f>
         <v/>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>28347121.58999873</v>
-      </c>
-      <c r="N5" s="4" t="n">
-        <v>44784483.14999981</v>
-      </c>
-      <c r="O5" s="5">
+      <c r="M5" s="17" t="n">
+        <v>28347121.58999882</v>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>44784483.14999945</v>
+      </c>
+      <c r="O5" s="19">
         <f>N5/M5-1</f>
         <v/>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="17">
         <f>M5/B5</f>
         <v/>
       </c>
-      <c r="Q5" s="4">
+      <c r="Q5" s="17">
         <f>N5/C5</f>
         <v/>
       </c>
-      <c r="R5" s="17">
+      <c r="R5" s="33">
         <f>Q5/P5-1</f>
         <v/>
       </c>
-      <c r="S5" s="19">
+      <c r="S5" s="35">
         <f>G5/D5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>FSM</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="17" t="n">
         <v>42</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="17" t="n">
         <v>45</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="19">
         <f>C6/B6-1</f>
         <v/>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="17" t="n">
         <v>170555</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="17" t="n">
         <v>215773</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="19">
         <f>F6/E6-1</f>
         <v/>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="17">
         <f>E6/B6</f>
         <v/>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="17">
         <f>F6/C6</f>
         <v/>
       </c>
-      <c r="J6" s="17">
+      <c r="J6" s="33">
         <f>I6/H6-1</f>
         <v/>
       </c>
-      <c r="K6" s="18">
+      <c r="K6" s="34">
         <f>E6/B6/56</f>
         <v/>
       </c>
-      <c r="L6" s="18">
+      <c r="L6" s="34">
         <f>F6/C6/56</f>
         <v/>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>18127443.54999987</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>29458690.66000083</v>
-      </c>
-      <c r="O6" s="5">
+      <c r="M6" s="17" t="n">
+        <v>18127443.54999989</v>
+      </c>
+      <c r="N6" s="17" t="n">
+        <v>29458690.66000078</v>
+      </c>
+      <c r="O6" s="19">
         <f>N6/M6-1</f>
         <v/>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="17">
         <f>M6/B6</f>
         <v/>
       </c>
-      <c r="Q6" s="4">
+      <c r="Q6" s="17">
         <f>N6/C6</f>
         <v/>
       </c>
-      <c r="R6" s="17">
+      <c r="R6" s="33">
         <f>Q6/P6-1</f>
         <v/>
       </c>
-      <c r="S6" s="19">
+      <c r="S6" s="35">
         <f>G6/D6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>TOPLAM</t>
         </is>
@@ -1512,7 +2014,7 @@
         <f>SUM(C4:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="37">
         <f>C7/B7-1</f>
         <v/>
       </c>
@@ -1524,7 +2026,7 @@
         <f>SUM(F4:F6)</f>
         <v/>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="37">
         <f>F7/E7-1</f>
         <v/>
       </c>
@@ -1536,15 +2038,15 @@
         <f>F7/C7</f>
         <v/>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="25">
         <f>I7/H7-1</f>
         <v/>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="38">
         <f>E7/B7/56</f>
         <v/>
       </c>
-      <c r="L7" s="23">
+      <c r="L7" s="38">
         <f>F7/C7/56</f>
         <v/>
       </c>
@@ -1556,7 +2058,7 @@
         <f>SUM(N4:N6)</f>
         <v/>
       </c>
-      <c r="O7" s="22">
+      <c r="O7" s="37">
         <f>N7/M7-1</f>
         <v/>
       </c>
@@ -1568,31 +2070,31 @@
         <f>N7/C7</f>
         <v/>
       </c>
-      <c r="R7" s="8">
+      <c r="R7" s="25">
         <f>Q7/P7-1</f>
         <v/>
       </c>
-      <c r="S7" s="24">
+      <c r="S7" s="39">
         <f>G7/D7</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>Kadro = 31.08 itibariyla o magazada fiilen calisan TUM personel (sezonluk + kadrolu).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t>'Is / kadro' = urun adedi buyumesi / kadro buyumesi. 1,0x'in uzeri: is kadrodan hizli buyudu.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t>Ist. Yolu kadrosu en cok buyuyen magaza (50 -&gt; 61) ama ise ragmen kisi basi adedi de artti.</t>
         </is>
@@ -1604,7 +2106,1355 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Bes magaza kadro tablosu — as-of Igt &lt;= T AND (Ict IS NULL OR Ict &gt;= T)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Magaza</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu taban 30.06 · 2025</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu taban 30.06 · 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Taban Δ</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu 31.08 · 2025</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu 31.08 · 2026</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Sezon ici hareket 2025</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Sezon ici hareket 2026</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk 31.08 · 2025</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk 31.08 · 2026</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam 31.08 · 2025</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam 31.08 · 2026</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam Δ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>İST. YOLU</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="C4" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="D4" s="40">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="G4" s="40">
+        <f>E4-B4</f>
+        <v/>
+      </c>
+      <c r="H4" s="40">
+        <f>F4-C4</f>
+        <v/>
+      </c>
+      <c r="I4" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="J4" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="K4" s="17">
+        <f>E4+I4</f>
+        <v/>
+      </c>
+      <c r="L4" s="17">
+        <f>F4+J4</f>
+        <v/>
+      </c>
+      <c r="M4" s="40">
+        <f>L4-K4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>ÖZLÜCE</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="D5" s="40">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>41</v>
+      </c>
+      <c r="G5" s="40">
+        <f>E5-B5</f>
+        <v/>
+      </c>
+      <c r="H5" s="40">
+        <f>F5-C5</f>
+        <v/>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="17">
+        <f>E5+I5</f>
+        <v/>
+      </c>
+      <c r="L5" s="17">
+        <f>F5+J5</f>
+        <v/>
+      </c>
+      <c r="M5" s="40">
+        <f>L5-K5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>FSM</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="D6" s="40">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G6" s="40">
+        <f>E6-B6</f>
+        <v/>
+      </c>
+      <c r="H6" s="40">
+        <f>F6-C6</f>
+        <v/>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="K6" s="17">
+        <f>E6+I6</f>
+        <v/>
+      </c>
+      <c r="L6" s="17">
+        <f>F6+J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="40">
+        <f>L6-K6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>HEYKEL</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="D7" s="40">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="G7" s="40">
+        <f>E7-B7</f>
+        <v/>
+      </c>
+      <c r="H7" s="40">
+        <f>F7-C7</f>
+        <v/>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="K7" s="17">
+        <f>E7+I7</f>
+        <v/>
+      </c>
+      <c r="L7" s="17">
+        <f>F7+J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="40">
+        <f>L7-K7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>ŞURA</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="40">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" s="40">
+        <f>E8-B8</f>
+        <v/>
+      </c>
+      <c r="H8" s="40">
+        <f>F8-C8</f>
+        <v/>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="17">
+        <f>E8+I8</f>
+        <v/>
+      </c>
+      <c r="L8" s="17">
+        <f>F8+J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="40">
+        <f>L8-K8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="B9" s="21">
+        <f>SUM(B4:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="21">
+        <f>SUM(C4:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="30">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>SUM(E4:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>SUM(F4:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="41">
+        <f>E9-B9</f>
+        <v/>
+      </c>
+      <c r="H9" s="30">
+        <f>F9-C9</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>SUM(I4:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>SUM(J4:J8)</f>
+        <v/>
+      </c>
+      <c r="K9" s="21">
+        <f>E9+I9</f>
+        <v/>
+      </c>
+      <c r="L9" s="21">
+        <f>F9+J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="41">
+        <f>L9-K9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>TABAN FARKI (D kolonu, TOPLAM satiri) = patrona soylenen +14: kadrolu 139 -&gt; 153, 1 TEMMUZ'DAN ONCE olustu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>SEZON ICI HAREKET = kesim - taban. 2026'da -4; 2025'te de -4 -&gt; sezon icinde kadro buyutulmedi, iki yilin deseni ayni.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>Sayim TEK TABLO uzerinden (vw_PersonelDepartman). Onceki surumde perbilgi LEFT JOIN'i bir kisiyi iki kez saymis:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ozluce 31.08.2026 kadrolu 42 gorunuyordu, DOGRUSU 41 (teyit: KADRO 41 + SEZONLUK 13 = 54 kisi).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bu yuzden magaza toplami 150 degil 149; sezon ici hareket -3 degil -4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>Heykel ve Sura POS raporlamasinda yok -&gt; is hacmi sayfalarinda yer almaz, kadro tablosunda VARDIR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>KAPSAM: Lokasyon = MAGAZALAR. Cift gorevli 1 kisi (GM satinalma 'KITAP DISI S.A' + Heykel) bu</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   kapsamda GORUNMEZ. O kisi Heykel'e eklenirse taban 140 -&gt; 154, kesim 136 -&gt; 150 olur;</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   TABAN FARKI yine +14, SEZON ICI HAREKET yine -4. Yani cift gorev savunmayi DEGISTIRMIYOR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>Kaynak view anlik durumu tutar (kadro gecmisi yok): kisinin BUGUNKU lokasyon etiketi her iki yila</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   da uygulanir. Bu yuzden kapsam iki yilda tutarli, ama gecmis unvan/lokasyon degisimi izlenemez.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Bölüm bazında kadro — 31.08 kesimi, beş mağaza</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Bolum</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu 2025</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Kadrolu Δ</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk 2025</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk 2026</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk Δ</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam 2025</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam 2026</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Toplam Δ</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Sezonluk payi 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>YARDIMCI KİTAP</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" s="40">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="G4" s="40">
+        <f>F4-E4</f>
+        <v/>
+      </c>
+      <c r="H4" s="17">
+        <f>B4+E4</f>
+        <v/>
+      </c>
+      <c r="I4" s="17">
+        <f>C4+F4</f>
+        <v/>
+      </c>
+      <c r="J4" s="40">
+        <f>I4-H4</f>
+        <v/>
+      </c>
+      <c r="K4" s="42">
+        <f>IF(I4=0,"",F4/I4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>KIRTASİYE</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D5" s="40">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="G5" s="40">
+        <f>F5-E5</f>
+        <v/>
+      </c>
+      <c r="H5" s="17">
+        <f>B5+E5</f>
+        <v/>
+      </c>
+      <c r="I5" s="17">
+        <f>C5+F5</f>
+        <v/>
+      </c>
+      <c r="J5" s="40">
+        <f>I5-H5</f>
+        <v/>
+      </c>
+      <c r="K5" s="42">
+        <f>IF(I5=0,"",F5/I5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>KÜLTÜR</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="40">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="40">
+        <f>F6-E6</f>
+        <v/>
+      </c>
+      <c r="H6" s="17">
+        <f>B6+E6</f>
+        <v/>
+      </c>
+      <c r="I6" s="17">
+        <f>C6+F6</f>
+        <v/>
+      </c>
+      <c r="J6" s="40">
+        <f>I6-H6</f>
+        <v/>
+      </c>
+      <c r="K6" s="42">
+        <f>IF(I6=0,"",F6/I6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>KASA</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="40">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="40">
+        <f>F7-E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="17">
+        <f>B7+E7</f>
+        <v/>
+      </c>
+      <c r="I7" s="17">
+        <f>C7+F7</f>
+        <v/>
+      </c>
+      <c r="J7" s="40">
+        <f>I7-H7</f>
+        <v/>
+      </c>
+      <c r="K7" s="42">
+        <f>IF(I7=0,"",F7/I7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>ÇOCUK</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="40">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="40">
+        <f>F8-E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>B8+E8</f>
+        <v/>
+      </c>
+      <c r="I8" s="17">
+        <f>C8+F8</f>
+        <v/>
+      </c>
+      <c r="J8" s="40">
+        <f>I8-H8</f>
+        <v/>
+      </c>
+      <c r="K8" s="42">
+        <f>IF(I8=0,"",F8/I8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>OYUNCAK</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="40">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="40">
+        <f>F9-E9</f>
+        <v/>
+      </c>
+      <c r="H9" s="17">
+        <f>B9+E9</f>
+        <v/>
+      </c>
+      <c r="I9" s="17">
+        <f>C9+F9</f>
+        <v/>
+      </c>
+      <c r="J9" s="40">
+        <f>I9-H9</f>
+        <v/>
+      </c>
+      <c r="K9" s="42">
+        <f>IF(I9=0,"",F9/I9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>AKADEMİ</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="40">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="40">
+        <f>F10-E10</f>
+        <v/>
+      </c>
+      <c r="H10" s="17">
+        <f>B10+E10</f>
+        <v/>
+      </c>
+      <c r="I10" s="17">
+        <f>C10+F10</f>
+        <v/>
+      </c>
+      <c r="J10" s="40">
+        <f>I10-H10</f>
+        <v/>
+      </c>
+      <c r="K10" s="42">
+        <f>IF(I10=0,"",F10/I10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>MAĞAZA</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="40">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="40">
+        <f>F11-E11</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>B11+E11</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
+        <f>C11+F11</f>
+        <v/>
+      </c>
+      <c r="J11" s="40">
+        <f>I11-H11</f>
+        <v/>
+      </c>
+      <c r="K11" s="42">
+        <f>IF(I11=0,"",F11/I11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>MAL KABUL</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="40">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="40">
+        <f>F12-E12</f>
+        <v/>
+      </c>
+      <c r="H12" s="17">
+        <f>B12+E12</f>
+        <v/>
+      </c>
+      <c r="I12" s="17">
+        <f>C12+F12</f>
+        <v/>
+      </c>
+      <c r="J12" s="40">
+        <f>I12-H12</f>
+        <v/>
+      </c>
+      <c r="K12" s="42">
+        <f>IF(I12=0,"",F12/I12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>İDARİ İŞLER</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="40">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="40">
+        <f>F13-E13</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>B13+E13</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
+        <f>C13+F13</f>
+        <v/>
+      </c>
+      <c r="J13" s="40">
+        <f>I13-H13</f>
+        <v/>
+      </c>
+      <c r="K13" s="42">
+        <f>IF(I13=0,"",F13/I13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>ETKİNLİK</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="40">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="40">
+        <f>F14-E14</f>
+        <v/>
+      </c>
+      <c r="H14" s="17">
+        <f>B14+E14</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
+        <f>C14+F14</f>
+        <v/>
+      </c>
+      <c r="J14" s="40">
+        <f>I14-H14</f>
+        <v/>
+      </c>
+      <c r="K14" s="42">
+        <f>IF(I14=0,"",F14/I14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>ŞURA</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="40">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="40">
+        <f>F15-E15</f>
+        <v/>
+      </c>
+      <c r="H15" s="17">
+        <f>B15+E15</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>C15+F15</f>
+        <v/>
+      </c>
+      <c r="J15" s="40">
+        <f>I15-H15</f>
+        <v/>
+      </c>
+      <c r="K15" s="42">
+        <f>IF(I15=0,"",F15/I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>ÖN MUHASEBE</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="40">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="40">
+        <f>F16-E16</f>
+        <v/>
+      </c>
+      <c r="H16" s="17">
+        <f>B16+E16</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>C16+F16</f>
+        <v/>
+      </c>
+      <c r="J16" s="40">
+        <f>I16-H16</f>
+        <v/>
+      </c>
+      <c r="K16" s="42">
+        <f>IF(I16=0,"",F16/I16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>MUHASEBE</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="40">
+        <f>C17-B17</f>
+        <v/>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="40">
+        <f>F17-E17</f>
+        <v/>
+      </c>
+      <c r="H17" s="17">
+        <f>B17+E17</f>
+        <v/>
+      </c>
+      <c r="I17" s="17">
+        <f>C17+F17</f>
+        <v/>
+      </c>
+      <c r="J17" s="40">
+        <f>I17-H17</f>
+        <v/>
+      </c>
+      <c r="K17" s="42">
+        <f>IF(I17=0,"",F17/I17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>BİLGİ İŞLEM</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="40">
+        <f>C18-B18</f>
+        <v/>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="40">
+        <f>F18-E18</f>
+        <v/>
+      </c>
+      <c r="H18" s="17">
+        <f>B18+E18</f>
+        <v/>
+      </c>
+      <c r="I18" s="17">
+        <f>C18+F18</f>
+        <v/>
+      </c>
+      <c r="J18" s="40">
+        <f>I18-H18</f>
+        <v/>
+      </c>
+      <c r="K18" s="42">
+        <f>IF(I18=0,"",F18/I18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>KIYAFET</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="40">
+        <f>C19-B19</f>
+        <v/>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="40">
+        <f>F19-E19</f>
+        <v/>
+      </c>
+      <c r="H19" s="17">
+        <f>B19+E19</f>
+        <v/>
+      </c>
+      <c r="I19" s="17">
+        <f>C19+F19</f>
+        <v/>
+      </c>
+      <c r="J19" s="40">
+        <f>I19-H19</f>
+        <v/>
+      </c>
+      <c r="K19" s="42">
+        <f>IF(I19=0,"",F19/I19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>SUM(B4:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="21">
+        <f>SUM(C4:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="30">
+        <f>C20-B20</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>SUM(E4:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>SUM(F4:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="41">
+        <f>F20-E20</f>
+        <v/>
+      </c>
+      <c r="H20" s="21">
+        <f>B20+E20</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>C20+F20</f>
+        <v/>
+      </c>
+      <c r="J20" s="41">
+        <f>I20-H20</f>
+        <v/>
+      </c>
+      <c r="K20" s="43">
+        <f>IF(I20=0,"",F20/I20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>OKUNACAK NOKTA: yonetim (MAGAZA departmani) ve MAL KABUL BUYUMEDI — artis satis/kasa tarafinda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>Sezonluk payi yuksek bolumler (KIRTASIYE, YARDIMCI KITAP, KIYAFET) sezon yuku tasiyan reyonlar;</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   oradaki kisi artisi kalici kadro degil, Eylul sonunda tahliye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>Bolum = Zirve 'Departman' alani (reyon). Bir kisi tek bolumde sayilir; toplam kapsam sayimiyla mutabik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>Devir (turnover) bolum bazinda AYRI olculdu: en bozuk COCUK %179 · IDARI ISLER %183 · KASA %160;</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAGAZA (yonetim) %25 ve ayrilanin ortalama kidemi 4,7 yil -&gt; yonetim katmani stabil.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1621,139 +3471,139 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Kisi basi is — 4 yillik trend (uc POS magazasi, Ocak-Agustos kumulatif, Sinav haric)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Yil</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Kadrolu (31.08)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Urun adedi (Oca-Agu)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Adet / kisi</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Onceki yila gore</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="16" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="17" t="n">
         <v>60</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="17" t="n">
         <v>2064284.43</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="44">
         <f>C4/B4</f>
         <v/>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="16" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="17" t="n">
         <v>91</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="17" t="n">
         <v>2296833.43</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="44">
         <f>C5/B5</f>
         <v/>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="19">
         <f>D5/D4-1</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="16" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="17" t="n">
         <v>96</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="17" t="n">
         <v>2752385.04</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="44">
         <f>C6/B6</f>
         <v/>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="19">
         <f>D6/D5-1</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="16" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="17" t="n">
         <v>111</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="17" t="n">
         <v>3607308.91</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="44">
         <f>C7/B7</f>
         <v/>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="19">
         <f>D7/D6-1</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>2024 ATLAMASI: kadrolu 60 -&gt; 91, adet yalniz +%11 -&gt; kisi basi is -%27. Kadro sismesi 2024'te oldu.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>AMA 2023 verimliligi 'norm' DEGIL: 2023'te FSM kasada 0 kisi, Ozluce kasada 1 kisi vardi (eksik kadroyla calisma).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>2024 -&gt; 2026: kisi basi is +%28,8 toparlanma. Bu yil kadro +15 kisi buyurken kisi basi is de artti.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Bu sayfada kadro yalniz KADROLU (sezonluk haric) — yillar arasi sezonluk tahliye zamanlamasi kiyasi bozuyor.</t>
         </is>
@@ -1765,7 +3615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1784,105 +3634,105 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>"Buyume kurumsaldan geldi" itirazinin cevabi — Ocak-Agustos, uc POS magazasi</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Kanal</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Adet 2025</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Adet 2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Adet Δ%</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Ciro 2025 (KDV dahil)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>Ciro 2026 (KDV dahil)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Ciro Δ%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Magaza (perakende raf)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="17" t="n">
         <v>2752385.04</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="17" t="n">
         <v>3607308.91</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="19">
         <f>C4/B4-1</f>
         <v/>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>316059798.2201176</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>489433287.7801854</v>
-      </c>
-      <c r="G4" s="5">
+      <c r="E4" s="17" t="n">
+        <v>316059798.2202811</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>489433287.7802867</v>
+      </c>
+      <c r="G4" s="19">
         <f>F4/E4-1</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Sinav Okullari (kurumsal)</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="17" t="n">
         <v>33584</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="17" t="n">
         <v>21693</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="19">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>136108071.4499996</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>105575646.11</v>
-      </c>
-      <c r="G5" s="5">
+      <c r="E5" s="17" t="n">
+        <v>136108071.4499999</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>105575646.1100004</v>
+      </c>
+      <c r="G5" s="19">
         <f>F5/E5-1</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t>TOPLAM</t>
         </is>
@@ -1895,7 +3745,7 @@
         <f>SUM(C4:C5)</f>
         <v/>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="37">
         <f>C6/B6-1</f>
         <v/>
       </c>
@@ -1907,27 +3757,27 @@
         <f>SUM(F4:F5)</f>
         <v/>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="37">
         <f>F6/E6-1</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Sinav Okullari KUCULDU (adet -%35, ciro -%22). Buyumenin tamami magaza rafindan geldi.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Magaza tarafi kurumsal dususu de kapatti: toplam yine buyudu.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Sinav = Kategori3 'Sinav Okullari' + 'Sinav Kiyafet'; ayni POS belgesi icinde geldigi icin AYIKLANMASI zorunlu.</t>
         </is>
@@ -1938,7 +3788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1952,135 +3802,135 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Yontem ve kaynaklar</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>Baslik</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="46" t="inlineStr">
         <is>
           <t>Kişi başı iş hacmi — sezon 2026 vs 2025</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>Kesim tarihi</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>otomatik (veri sonu, okul-hizalı pencerede)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>Pencere</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="46" t="inlineStr">
         <is>
           <t>Okul açılışına hizalı: 2025 açılış 20250908, 2026 açılış 20260914; gün ofseti -69..-14 = her iki yıl 56 gün</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="45" t="inlineStr">
         <is>
           <t>Kadro kaynagi</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>Zirve BKM_GENEL.dbo.vw_PersonelDepartman — as-of Igt &lt;= T AND (Ict IS NULL OR Ict &gt;= T), sp_PersonelKarsilastirma_Ozet ile birebir</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>Is hacmi kaynagi</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="46" t="inlineStr">
         <is>
           <t>DerinSIS irs/irsAyr eTip=100 (POS satışı), Sınav Okulları/Kıyafet hariç, iade netlenmiş</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="45" t="inlineStr">
         <is>
           <t>Cekirdek SQL</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="46" t="inlineStr">
         <is>
           <t>sorgular/2026-09-02-kadro-vs-is-hacmi-savunma.sql (blok 11)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Dikkat edilecekler</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>• Ürün adedi enflasyondan bağımsız — kadro kıyasında birincil ölçüt. Ciro ikincil (fiyat endeksi +%19,8, Fisher, eşleşen ürün).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>• Kıyas okul açılışına hizalı yapılır. Takvim tarihine göre kıyas 2026'da yapay düşüş gösterir: açılış 8 Eylül 2025'ten 14 Eylül 2026'ya, 6 gün kaydı.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>• İş hacmi EncoreMerkez POS'tan DEĞİL DerinSIS'ten alınır: POS Temmuz 2025'te değişti (ENPOS → EncoreMerkez), EncoreMerkez'in 2025 tabanı eksik.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>• Heykel ve Şura POS raporlamasında yok — mağaza sayfası üç POS mağazası (FSM · Özlüce · İst. Yolu). Beş mağaza kadro hareketi Özet'te ayrı.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>• Kadro = o tarihte fiilen çalışan kişi (sezonluk + kadrolu). Kişi başı oranlar kasiyer değil TÜM mağaza kadrosu üzerinden.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="48" t="inlineStr">
         <is>
           <t>• Fiş sayısı bu kaynakta yok: eTip 100 günlük özet belgedir (bir gün = bir belge).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>• Kıdem → verimlilik testi NEGATİF çıktı: aynı kasiyerin öğrenme eğrisi düz (220 → 256 → 242 fiş/gün), mağaza kıdem sıralaması verimlilikle uyuşmuyor. 'Tecrübeli 1 kişi = acemi 3 kişi' iddiası bu veriyle savunulamaz.</t>
         </is>

</xml_diff>

<commit_message>
feat(bkm): bölüm bazlı norm açığı da engelli-dışı kurala getirildi
Kullanıcı: "bölüm dağılımını da çek aynı kurala getir".

Engelli bölüm dağılımı canlı ölçüldü (dört norm mağazası, 31.08 as-of): KIRTASİYE 2 · MAL KABUL 1.
Bölüm tablosunda artık operasyonel kadrolu = kadrolu − engelli; ayrı "Engelli (norm dışı)" kolonu
şeffaflık için duruyor. ETKİNLİK normda tanımlı olmadığı için tablodan çıkarılıp en alta
"norm dışı" satırı olarak (krem zemin) alındı, toplamlara girmiyor.

Etki: bölüm bazlı açık 15 → 17 (Kırtasiye ve Mal Kabul artık açıkta; Kırtasiye önce +1 fazla
görünüyordu). Fazla yalnız Yardımcı Kitap +3. Mağaza bazlı açık da operasyonel hale getirildi
(14) — "neden bölüm toplamından büyük" kutusu 17 vs 14 ile güncellendi.

Artık üç katman aynı kuralı kullanıyor: yönetici özeti (−28), mağaza detayı (kadrolu −14 ·
sezonluk −14), bölüm detayı (açık 17 · fazla 3).

Denetçi: ✓ ihlal yok.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/briefings/sezon-kadro-20260902/verimlilik-2026.xlsx
+++ b/briefings/sezon-kadro-20260902/verimlilik-2026.xlsx
@@ -1517,14 +1517,14 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Kültür</t>
+          <t>Mağaza</t>
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D13" s="55" t="n">
         <v>2</v>
@@ -1535,20 +1535,20 @@
         </is>
       </c>
       <c r="F13" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>Mağaza</t>
+          <t>İdari̇ İşler</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D14" s="55" t="n">
         <v>2</v>
@@ -1565,14 +1565,14 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>İdari̇ İşler</t>
+          <t>Kültür</t>
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D15" s="55" t="n">
         <v>2</v>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="F15" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1637,14 +1637,14 @@
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Oyun Alani</t>
+          <t>Akademi̇</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D18" s="55" t="n">
         <v>1</v>
@@ -1661,14 +1661,14 @@
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Akademi̇</t>
+          <t>Oyun Alani</t>
         </is>
       </c>
       <c r="B19" s="17" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D19" s="55" t="n">
         <v>1</v>
@@ -1685,101 +1685,99 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Kiyafet</t>
+          <t>Mal Kabul</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="17" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="D20" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="F20" s="17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Kirtasi̇ye</t>
+          <t>Oyuncak</t>
         </is>
       </c>
       <c r="B21" s="17" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="17" t="n">
-        <v>1</v>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F21" s="17" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Mal Kabul</t>
+          <t>Yardimci Ki̇tap</t>
         </is>
       </c>
       <c r="B22" s="17" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C22" s="17" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="17" t="n">
+        <v>3</v>
       </c>
       <c r="F22" s="17" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Yardimci Ki̇tap</t>
+          <t>Kirtasi̇ye</t>
         </is>
       </c>
       <c r="B23" s="17" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="D23" s="17" t="inlineStr">
+        <v>23</v>
+      </c>
+      <c r="D23" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n">
-        <v>3</v>
-      </c>
       <c r="F23" s="17" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -1809,14 +1807,14 @@
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Oyuncak</t>
+          <t>Kiyafet</t>
         </is>
       </c>
       <c r="B25" s="17" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
@@ -1829,7 +1827,7 @@
         </is>
       </c>
       <c r="F25" s="17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -1842,13 +1840,13 @@
         <v>145</v>
       </c>
       <c r="C26" s="21" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D26" s="21" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F26" s="21" t="n">
         <v>58</v>
@@ -1857,7 +1855,7 @@
     <row r="28">
       <c r="A28" s="32" t="inlineStr">
         <is>
-          <t>⚠ BOLUM acigi (15) MAGAZA acigindan (11) BUYUK: magaza icinde bir bolumun fazlasi baska bolumun acigini maskeler.</t>
+          <t>⚠ BOLUM acigi (17) MAGAZA acigindan (11) BUYUK: magaza icinde bir bolumun fazlasi baska bolumun acigini maskeler.</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2198,7 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>66929723.56999852</v>
+        <v>66929723.56999993</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>114687785.58</v>
@@ -2221,10 +2219,10 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>71837429.11999343</v>
+        <v>71837429.12000012</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>122601380.8499947</v>
+        <v>122601380.8500001</v>
       </c>
       <c r="D10" s="18">
         <f>C10-B10</f>
@@ -2758,10 +2756,10 @@
         <v/>
       </c>
       <c r="M4" s="17" t="n">
-        <v>20455158.42999981</v>
+        <v>20455158.42999999</v>
       </c>
       <c r="N4" s="17" t="n">
-        <v>40444611.76999976</v>
+        <v>40444611.77</v>
       </c>
       <c r="O4" s="19">
         <f>N4/M4-1</f>
@@ -2831,10 +2829,10 @@
         <v/>
       </c>
       <c r="M5" s="17" t="n">
-        <v>28347121.58999882</v>
+        <v>28347121.58999996</v>
       </c>
       <c r="N5" s="17" t="n">
-        <v>44784483.14999945</v>
+        <v>44784483.15000006</v>
       </c>
       <c r="O5" s="19">
         <f>N5/M5-1</f>
@@ -2904,10 +2902,10 @@
         <v/>
       </c>
       <c r="M6" s="17" t="n">
-        <v>18127443.54999989</v>
+        <v>18127443.54999998</v>
       </c>
       <c r="N6" s="17" t="n">
-        <v>29458690.66000078</v>
+        <v>29458690.65999999</v>
       </c>
       <c r="O6" s="19">
         <f>N6/M6-1</f>
@@ -4504,10 +4502,10 @@
         <v/>
       </c>
       <c r="F4" s="34" t="n">
-        <v>18.5043249700029</v>
+        <v>18.50432496999891</v>
       </c>
       <c r="G4" s="34" t="n">
-        <v>32.38086690000142</v>
+        <v>32.38086689999964</v>
       </c>
       <c r="H4" s="44">
         <f>G4/F4-1</f>
@@ -4524,7 +4522,7 @@
         <v/>
       </c>
       <c r="L4" s="19" t="n">
-        <v>0.3747245332289066</v>
+        <v>0.3747245332273854</v>
       </c>
       <c r="M4" s="45" t="n">
         <v>3</v>
@@ -4552,10 +4550,10 @@
         <v/>
       </c>
       <c r="F5" s="34" t="n">
-        <v>10.02370844000001</v>
+        <v>10.02370843999998</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>15.50422909000001</v>
+        <v>15.50422908999993</v>
       </c>
       <c r="H5" s="44">
         <f>G5/F5-1</f>
@@ -4572,7 +4570,7 @@
         <v/>
       </c>
       <c r="L5" s="19" t="n">
-        <v>0.5770282964720019</v>
+        <v>0.5770282964720066</v>
       </c>
       <c r="M5" s="45" t="n">
         <v>-1</v>
@@ -4600,10 +4598,10 @@
         <v/>
       </c>
       <c r="F6" s="34" t="n">
-        <v>14.49106598999973</v>
+        <v>14.49106599000013</v>
       </c>
       <c r="G6" s="34" t="n">
-        <v>23.14058788999986</v>
+        <v>23.14058788999988</v>
       </c>
       <c r="H6" s="44">
         <f>G6/F6-1</f>
@@ -4620,7 +4618,7 @@
         <v/>
       </c>
       <c r="L6" s="19" t="n">
-        <v>0.4921459875658136</v>
+        <v>0.4921459875659902</v>
       </c>
       <c r="M6" s="45" t="n">
         <v>1</v>
@@ -4668,7 +4666,7 @@
         <v/>
       </c>
       <c r="L7" s="19" t="n">
-        <v>1.797673394233621</v>
+        <v>1.797673394233624</v>
       </c>
       <c r="M7" s="40" t="inlineStr">
         <is>
@@ -4701,7 +4699,7 @@
         <v>11.13631268</v>
       </c>
       <c r="G8" s="34" t="n">
-        <v>16.74884972000006</v>
+        <v>16.74884971999999</v>
       </c>
       <c r="H8" s="44">
         <f>G8/F8-1</f>
@@ -4718,7 +4716,7 @@
         <v/>
       </c>
       <c r="L8" s="19" t="n">
-        <v>0.6655996445023109</v>
+        <v>0.6655996445022587</v>
       </c>
       <c r="M8" s="45" t="n">
         <v>1</v>
@@ -4746,10 +4744,10 @@
         <v/>
       </c>
       <c r="F9" s="34" t="n">
-        <v>1.475290260000008</v>
+        <v>1.47529026</v>
       </c>
       <c r="G9" s="34" t="n">
-        <v>2.616103030000003</v>
+        <v>2.616103029999998</v>
       </c>
       <c r="H9" s="44">
         <f>G9/F9-1</f>
@@ -4766,7 +4764,7 @@
         <v/>
       </c>
       <c r="L9" s="19" t="n">
-        <v>1.258006023303491</v>
+        <v>1.258006023303307</v>
       </c>
       <c r="M9" s="40" t="inlineStr">
         <is>
@@ -4796,10 +4794,10 @@
         <v/>
       </c>
       <c r="F10" s="34" t="n">
-        <v>11.66512254</v>
+        <v>11.66512254000002</v>
       </c>
       <c r="G10" s="34" t="n">
-        <v>22.35794457999994</v>
+        <v>22.35794457999999</v>
       </c>
       <c r="H10" s="44">
         <f>G10/F10-1</f>
@@ -4816,7 +4814,7 @@
         <v/>
       </c>
       <c r="L10" s="19" t="n">
-        <v>0.4621370345582292</v>
+        <v>0.4621370345582057</v>
       </c>
       <c r="M10" s="45" t="n">
         <v>6</v>
@@ -4847,7 +4845,7 @@
         <v>0.69211733</v>
       </c>
       <c r="G11" s="34" t="n">
-        <v>1.187673780000001</v>
+        <v>1.187673779999999</v>
       </c>
       <c r="H11" s="44">
         <f>G11/F11-1</f>
@@ -4864,7 +4862,7 @@
         <v/>
       </c>
       <c r="L11" s="19" t="n">
-        <v>0.4636366398909368</v>
+        <v>0.4636366398909304</v>
       </c>
       <c r="M11" s="40" t="inlineStr">
         <is>
@@ -4894,10 +4892,10 @@
         <v/>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.942142249999998</v>
+        <v>1.942142250000001</v>
       </c>
       <c r="G12" s="34" t="n">
-        <v>6.643827519999992</v>
+        <v>6.643827520000001</v>
       </c>
       <c r="H12" s="44">
         <f>G12/F12-1</f>
@@ -4914,7 +4912,7 @@
         <v/>
       </c>
       <c r="L12" s="19" t="n">
-        <v>1.769093453522593</v>
+        <v>1.769093453522601</v>
       </c>
       <c r="M12" s="45" t="n">
         <v>2</v>
@@ -4945,7 +4943,7 @@
         <v>0.2846255699999998</v>
       </c>
       <c r="G13" s="34" t="n">
-        <v>0.4203621899999997</v>
+        <v>0.4203621899999998</v>
       </c>
       <c r="H13" s="44">
         <f>G13/F13-1</f>
@@ -4962,7 +4960,7 @@
         <v/>
       </c>
       <c r="L13" s="19" t="n">
-        <v>0.5224217348514228</v>
+        <v>0.5224217348514244</v>
       </c>
       <c r="M13" s="40" t="inlineStr">
         <is>
@@ -4992,10 +4990,10 @@
         <v/>
       </c>
       <c r="F14" s="34" t="n">
-        <v>1.257655950000001</v>
+        <v>1.25765595</v>
       </c>
       <c r="G14" s="34" t="n">
-        <v>0.9961937400000004</v>
+        <v>0.9961937400000002</v>
       </c>
       <c r="H14" s="44">
         <f>G14/F14-1</f>
@@ -5012,7 +5010,7 @@
         <v/>
       </c>
       <c r="L14" s="19" t="n">
-        <v>0.4008427609025746</v>
+        <v>0.4008427609025693</v>
       </c>
       <c r="M14" s="40" t="inlineStr">
         <is>
@@ -5042,10 +5040,10 @@
         <v/>
       </c>
       <c r="F15" s="34" t="n">
-        <v>0.2656298399999997</v>
+        <v>0.2656298400000003</v>
       </c>
       <c r="G15" s="34" t="n">
-        <v>0.3784858199999995</v>
+        <v>0.37848582</v>
       </c>
       <c r="H15" s="44">
         <f>G15/F15-1</f>
@@ -5062,7 +5060,7 @@
         <v/>
       </c>
       <c r="L15" s="19" t="n">
-        <v>0.4999858989104862</v>
+        <v>0.4999858989104888</v>
       </c>
       <c r="M15" s="40" t="inlineStr">
         <is>
@@ -5240,10 +5238,10 @@
         <v/>
       </c>
       <c r="E4" s="34" t="n">
-        <v>33.37095816000334</v>
+        <v>33.37095815999883</v>
       </c>
       <c r="F4" s="34" t="n">
-        <v>49.92745520000055</v>
+        <v>49.92745519999968</v>
       </c>
       <c r="G4" s="44">
         <f>F4/E4-1</f>
@@ -5267,10 +5265,10 @@
         <v/>
       </c>
       <c r="E5" s="34" t="n">
-        <v>32.14602051000339</v>
+        <v>32.14602050999881</v>
       </c>
       <c r="F5" s="34" t="n">
-        <v>55.81932909000084</v>
+        <v>55.81932908999958</v>
       </c>
       <c r="G5" s="44">
         <f>F5/E5-1</f>
@@ -5294,10 +5292,10 @@
         <v/>
       </c>
       <c r="E6" s="34" t="n">
-        <v>61.34527556000126</v>
+        <v>61.34527556000244</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>78.15309667999897</v>
+        <v>78.15309668000015</v>
       </c>
       <c r="G6" s="44">
         <f>F6/E6-1</f>
@@ -5776,10 +5774,10 @@
         <v/>
       </c>
       <c r="E4" s="17" t="n">
-        <v>316059798.2201092</v>
+        <v>316059798.2198316</v>
       </c>
       <c r="F4" s="17" t="n">
-        <v>489433287.7801834</v>
+        <v>489433287.7799246</v>
       </c>
       <c r="G4" s="19">
         <f>F4/E4-1</f>
@@ -5803,10 +5801,10 @@
         <v/>
       </c>
       <c r="E5" s="17" t="n">
-        <v>136108071.4499997</v>
+        <v>136108071.45</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>105575646.1100001</v>
+        <v>105575646.11</v>
       </c>
       <c r="G5" s="19">
         <f>F5/E5-1</f>

</xml_diff>